<commit_message>
Update activities as of 2026-03-06
</commit_message>
<xml_diff>
--- a/data/portfolio_activity.xlsx
+++ b/data/portfolio_activity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johanrosa/Desktop/web_development/personal/finance_portfolio/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2018001\work_desktop\_personal\finance_portfolio\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E8AAEDD-FE80-1B4B-9F32-586F9D3D2E85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B624C6E8-36BD-4F8F-93E3-91426187A02F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{22981F44-200C-FA48-B0C7-1CB3C862DEAA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{22981F44-200C-FA48-B0C7-1CB3C862DEAA}"/>
   </bookViews>
   <sheets>
     <sheet name="logs" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="59">
   <si>
     <t>date</t>
   </si>
@@ -225,7 +225,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="0.00000"/>
+    <numFmt numFmtId="166" formatCode="0.00000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -283,7 +283,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -620,18 +620,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64184D08-D91B-1043-AEE3-17C45FED0F30}">
-  <dimension ref="A1:F128"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F135"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.1640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15.125" style="1" customWidth="1"/>
     <col min="2" max="2" width="18.5" style="2" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="15.625" style="6" customWidth="1"/>
     <col min="4" max="4" width="21.5" style="6" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" style="6"/>
-    <col min="6" max="6" width="10.83203125" style="2"/>
+    <col min="5" max="5" width="10.875" style="6"/>
+    <col min="6" max="6" width="10.875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -651,7 +651,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>45903.43472222222</v>
       </c>
@@ -672,7 +672,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>45903.435416666667</v>
       </c>
@@ -693,7 +693,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>45903.436111111114</v>
       </c>
@@ -714,7 +714,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>45903.436805555553</v>
       </c>
@@ -735,7 +735,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>45903.438194444447</v>
       </c>
@@ -756,7 +756,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>45903.438888888886</v>
       </c>
@@ -777,7 +777,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>45903.418749999997</v>
       </c>
@@ -798,7 +798,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>45903.445138888892</v>
       </c>
@@ -819,7 +819,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>45903.445833333331</v>
       </c>
@@ -839,7 +839,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>45903.448611111111</v>
       </c>
@@ -860,7 +860,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>45903.455555555556</v>
       </c>
@@ -881,7 +881,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>45903.463888888888</v>
       </c>
@@ -902,7 +902,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>45903.46597222222</v>
       </c>
@@ -923,7 +923,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>45903.467361111114</v>
       </c>
@@ -944,7 +944,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>45903.46875</v>
       </c>
@@ -965,7 +965,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>45903.470138888886</v>
       </c>
@@ -986,7 +986,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>45903.474999999999</v>
       </c>
@@ -1007,7 +1007,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>45903.476388888892</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>45903.479861111111</v>
       </c>
@@ -1049,7 +1049,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>45903.480555555558</v>
       </c>
@@ -1070,7 +1070,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>45903.493750000001</v>
       </c>
@@ -1091,7 +1091,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>45903.494444444441</v>
       </c>
@@ -1112,7 +1112,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>45903.494444444441</v>
       </c>
@@ -1133,7 +1133,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>45903.495138888888</v>
       </c>
@@ -1154,7 +1154,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>45903.504861111112</v>
       </c>
@@ -1175,7 +1175,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>45904.404861111114</v>
       </c>
@@ -1196,7 +1196,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>45904.406944444447</v>
       </c>
@@ -1217,7 +1217,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>45904.407638888886</v>
       </c>
@@ -1238,7 +1238,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>45904.412499999999</v>
       </c>
@@ -1259,7 +1259,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>45904.414583333331</v>
       </c>
@@ -1280,7 +1280,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>45904.418749999997</v>
       </c>
@@ -1301,7 +1301,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>45905.408333333333</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>45908.665277777778</v>
       </c>
@@ -1343,7 +1343,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>45909.415277777778</v>
       </c>
@@ -1364,7 +1364,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>45909.418055555558</v>
       </c>
@@ -1385,7 +1385,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>45909.427083333336</v>
       </c>
@@ -1406,7 +1406,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>45909.427777777775</v>
       </c>
@@ -1427,7 +1427,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>45909.431250000001</v>
       </c>
@@ -1448,7 +1448,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>45909.43472222222</v>
       </c>
@@ -1469,7 +1469,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>45909.439583333333</v>
       </c>
@@ -1490,7 +1490,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>45909.449305555558</v>
       </c>
@@ -1511,7 +1511,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>45909.449305555558</v>
       </c>
@@ -1532,7 +1532,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>45910</v>
       </c>
@@ -1553,7 +1553,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>45910</v>
       </c>
@@ -1574,7 +1574,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>45911</v>
       </c>
@@ -1595,7 +1595,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>45911</v>
       </c>
@@ -1616,7 +1616,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>45912</v>
       </c>
@@ -1637,7 +1637,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>45912</v>
       </c>
@@ -1658,7 +1658,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>45912</v>
       </c>
@@ -1679,7 +1679,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>45912</v>
       </c>
@@ -1700,7 +1700,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>45923</v>
       </c>
@@ -1721,7 +1721,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>45923</v>
       </c>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>45923</v>
       </c>
@@ -1763,7 +1763,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>45923</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>45923</v>
       </c>
@@ -1805,7 +1805,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>45923</v>
       </c>
@@ -1826,7 +1826,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>45924</v>
       </c>
@@ -1847,7 +1847,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>45924</v>
       </c>
@@ -1868,7 +1868,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>45929</v>
       </c>
@@ -1889,7 +1889,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>45937</v>
       </c>
@@ -1910,7 +1910,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>45937</v>
       </c>
@@ -1931,7 +1931,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>45937</v>
       </c>
@@ -1952,7 +1952,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>45937.40625</v>
       </c>
@@ -1973,7 +1973,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>45937.462500000001</v>
       </c>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>45937.465277777781</v>
       </c>
@@ -2015,7 +2015,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>45938.413194444445</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>45939.417361111111</v>
       </c>
@@ -2055,7 +2055,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>45943.410416666666</v>
       </c>
@@ -2075,7 +2075,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>45943.411805555559</v>
       </c>
@@ -2095,7 +2095,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>45943.412499999999</v>
       </c>
@@ -2115,7 +2115,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>45943.413194444445</v>
       </c>
@@ -2135,7 +2135,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>45943.415277777778</v>
       </c>
@@ -2155,7 +2155,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>45943.417361111111</v>
       </c>
@@ -2175,7 +2175,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>45946.399305555555</v>
       </c>
@@ -2195,7 +2195,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>45957.457638888889</v>
       </c>
@@ -2215,7 +2215,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>45957.459722222222</v>
       </c>
@@ -2235,7 +2235,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>45957.460416666669</v>
       </c>
@@ -2255,7 +2255,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>45957.462500000001</v>
       </c>
@@ -2275,7 +2275,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>45957.463194444441</v>
       </c>
@@ -2295,7 +2295,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>45957.463888888888</v>
       </c>
@@ -2315,7 +2315,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>45957.464583333334</v>
       </c>
@@ -2335,7 +2335,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>45957.464583333334</v>
       </c>
@@ -2355,7 +2355,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>45957.470833333333</v>
       </c>
@@ -2375,7 +2375,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>45957.470833333333</v>
       </c>
@@ -2395,7 +2395,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>45957.47152777778</v>
       </c>
@@ -2415,7 +2415,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>45958.512499999997</v>
       </c>
@@ -2435,7 +2435,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>45958.515277777777</v>
       </c>
@@ -2455,7 +2455,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>45958.517361111109</v>
       </c>
@@ -2475,7 +2475,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>45958.520138888889</v>
       </c>
@@ -2495,7 +2495,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>45958.522222222222</v>
       </c>
@@ -2515,7 +2515,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <v>45958.522222222222</v>
       </c>
@@ -2535,7 +2535,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>45958.529166666667</v>
       </c>
@@ -2555,7 +2555,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>45965.642361111109</v>
       </c>
@@ -2575,7 +2575,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
         <v>45974.67291666667</v>
       </c>
@@ -2595,7 +2595,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>46002.439583333333</v>
       </c>
@@ -2615,7 +2615,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>46002.443749999999</v>
       </c>
@@ -2635,7 +2635,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>46002.446527777778</v>
       </c>
@@ -2655,7 +2655,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>46008.648611111108</v>
       </c>
@@ -2675,7 +2675,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>46008.650694444441</v>
       </c>
@@ -2695,7 +2695,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>46020.463888888888</v>
       </c>
@@ -2715,7 +2715,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
         <v>46021.472916666666</v>
       </c>
@@ -2735,7 +2735,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
         <v>46027.567361111112</v>
       </c>
@@ -2755,7 +2755,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>46027.568055555559</v>
       </c>
@@ -2775,7 +2775,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
         <v>46027.568749999999</v>
       </c>
@@ -2795,7 +2795,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
         <v>46029.449305555558</v>
       </c>
@@ -2815,7 +2815,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
         <v>46034.47152777778</v>
       </c>
@@ -2835,7 +2835,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="1">
         <v>46034.47152777778</v>
       </c>
@@ -2855,7 +2855,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
         <v>46035.44027777778</v>
       </c>
@@ -2875,7 +2875,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
         <v>46035.441666666666</v>
       </c>
@@ -2895,7 +2895,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
         <v>46036.448611111111</v>
       </c>
@@ -2915,7 +2915,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
         <v>46042.441666666666</v>
       </c>
@@ -2935,7 +2935,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="1">
         <v>46042.44027777778</v>
       </c>
@@ -2955,7 +2955,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
         <v>46042.45</v>
       </c>
@@ -2975,7 +2975,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="1">
         <v>46044.496527777781</v>
       </c>
@@ -2996,7 +2996,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
         <v>46044.496527777781</v>
       </c>
@@ -3016,7 +3016,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
         <v>46044.49722222222</v>
       </c>
@@ -3036,7 +3036,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
         <v>46045.445833333331</v>
       </c>
@@ -3056,7 +3056,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
         <v>46045.493055555555</v>
       </c>
@@ -3076,7 +3076,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
         <v>46048.572222222225</v>
       </c>
@@ -3096,7 +3096,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
         <v>46049.448611111111</v>
       </c>
@@ -3116,7 +3116,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" s="1">
         <v>46050.563888888886</v>
       </c>
@@ -3136,7 +3136,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
         <v>46059</v>
       </c>
@@ -3156,7 +3156,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" s="1">
         <v>46055.650694444441</v>
       </c>
@@ -3176,7 +3176,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" s="1">
         <v>46055.652083333334</v>
       </c>
@@ -3196,7 +3196,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" s="1">
         <v>46083.456250000003</v>
       </c>
@@ -3216,7 +3216,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="1">
         <v>46086</v>
       </c>
@@ -3236,7 +3236,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
         <v>46002</v>
       </c>
@@ -3254,6 +3254,146 @@
       </c>
       <c r="F128" s="2" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A129" s="1">
+        <v>46087</v>
+      </c>
+      <c r="B129" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C129" s="6">
+        <v>599.1</v>
+      </c>
+      <c r="D129" s="6">
+        <v>299.41000000000003</v>
+      </c>
+      <c r="E129" s="6">
+        <v>2.0009399999999999</v>
+      </c>
+      <c r="F129" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A130" s="1">
+        <v>46087</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C130" s="6">
+        <v>467.44</v>
+      </c>
+      <c r="D130" s="6">
+        <v>45.39</v>
+      </c>
+      <c r="E130" s="6">
+        <v>10.297129999999999</v>
+      </c>
+      <c r="F130" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A131" s="1">
+        <v>46087</v>
+      </c>
+      <c r="B131" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C131" s="6">
+        <v>333.26</v>
+      </c>
+      <c r="D131" s="6">
+        <v>16.579999999999998</v>
+      </c>
+      <c r="E131" s="6">
+        <v>20.037700000000001</v>
+      </c>
+      <c r="F131" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A132" s="1">
+        <v>46087</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C132" s="6">
+        <v>525.9</v>
+      </c>
+      <c r="D132" s="6">
+        <v>59.68</v>
+      </c>
+      <c r="E132" s="6">
+        <v>8.8120799999999999</v>
+      </c>
+      <c r="F132" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A133" s="1">
+        <v>46087</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C133" s="6">
+        <v>462.97</v>
+      </c>
+      <c r="D133" s="6">
+        <v>81.02</v>
+      </c>
+      <c r="E133" s="6">
+        <v>5.7142799999999996</v>
+      </c>
+      <c r="F133" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A134" s="1">
+        <v>46087</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C134" s="6">
+        <v>291.45999999999998</v>
+      </c>
+      <c r="D134" s="6">
+        <v>80.78</v>
+      </c>
+      <c r="E134" s="6">
+        <v>3.60785</v>
+      </c>
+      <c r="F134" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A135" s="1">
+        <v>46087</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C135" s="6">
+        <v>222.54</v>
+      </c>
+      <c r="D135" s="6">
+        <v>20.58</v>
+      </c>
+      <c r="E135" s="6">
+        <v>10.81081</v>
+      </c>
+      <c r="F135" s="2" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Activities as of 2026-03-09
</commit_message>
<xml_diff>
--- a/data/portfolio_activity.xlsx
+++ b/data/portfolio_activity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2018001\work_desktop\_personal\finance_portfolio\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B624C6E8-36BD-4F8F-93E3-91426187A02F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4836B82-EE96-45B7-8CD4-796BBD814446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{22981F44-200C-FA48-B0C7-1CB3C862DEAA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="61">
   <si>
     <t>date</t>
   </si>
@@ -216,6 +216,12 @@
   </si>
   <si>
     <t>VDE</t>
+  </si>
+  <si>
+    <t>VIST</t>
+  </si>
+  <si>
+    <t>YPF</t>
   </si>
 </sst>
 </file>
@@ -620,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64184D08-D91B-1043-AEE3-17C45FED0F30}">
-  <dimension ref="A1:F135"/>
+  <dimension ref="A1:F139"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.125" style="1" customWidth="1"/>
@@ -3396,6 +3402,86 @@
         <v>38</v>
       </c>
     </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A136" s="1">
+        <v>46090</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C136" s="6">
+        <v>790.6</v>
+      </c>
+      <c r="D136" s="6">
+        <v>56.79</v>
+      </c>
+      <c r="E136" s="6">
+        <v>13.9215</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A137" s="1">
+        <v>46090</v>
+      </c>
+      <c r="B137" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C137" s="6">
+        <v>788</v>
+      </c>
+      <c r="D137" s="6">
+        <v>116.55</v>
+      </c>
+      <c r="E137" s="6">
+        <v>6.7617500000000001</v>
+      </c>
+      <c r="F137" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A138" s="1">
+        <v>46090</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C138" s="6">
+        <v>500</v>
+      </c>
+      <c r="D138" s="6">
+        <v>63.36</v>
+      </c>
+      <c r="E138" s="6">
+        <v>7.89</v>
+      </c>
+      <c r="F138" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A139" s="1">
+        <v>46090</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C139" s="6">
+        <v>500</v>
+      </c>
+      <c r="D139" s="6">
+        <v>37.89</v>
+      </c>
+      <c r="E139" s="6">
+        <v>13.19</v>
+      </c>
+      <c r="F139" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F128" xr:uid="{64184D08-D91B-1043-AEE3-17C45FED0F30}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update activities as of 2026-03-12
</commit_message>
<xml_diff>
--- a/data/portfolio_activity.xlsx
+++ b/data/portfolio_activity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johanrosa/Desktop/web_development/personal/finance_portfolio/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2018001\work_desktop\_personal\finance_portfolio\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{228B155B-5321-DC43-AA95-FE664358C160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DC93EB0-C50D-495B-BE81-6E7968941840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15720" xr2:uid="{22981F44-200C-FA48-B0C7-1CB3C862DEAA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{22981F44-200C-FA48-B0C7-1CB3C862DEAA}"/>
   </bookViews>
   <sheets>
     <sheet name="logs" sheetId="1" r:id="rId1"/>
@@ -630,17 +630,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64184D08-D91B-1043-AEE3-17C45FED0F30}">
   <dimension ref="A1:F146"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.1640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15.125" style="1" customWidth="1"/>
     <col min="2" max="2" width="18.5" style="2" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="15.625" style="6" customWidth="1"/>
     <col min="4" max="4" width="21.5" style="6" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" style="6"/>
-    <col min="6" max="6" width="10.83203125" style="2"/>
+    <col min="5" max="5" width="10.875" style="6"/>
+    <col min="6" max="6" width="10.875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -660,7 +660,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>45903.43472222222</v>
       </c>
@@ -681,7 +681,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>45903.435416666667</v>
       </c>
@@ -702,7 +702,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>45903.436111111114</v>
       </c>
@@ -723,7 +723,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>45903.436805555553</v>
       </c>
@@ -744,7 +744,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>45903.438194444447</v>
       </c>
@@ -765,7 +765,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>45903.438888888886</v>
       </c>
@@ -786,7 +786,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>45903.418749999997</v>
       </c>
@@ -807,7 +807,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>45903.445138888892</v>
       </c>
@@ -828,7 +828,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>45903.445833333331</v>
       </c>
@@ -848,7 +848,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>45903.448611111111</v>
       </c>
@@ -869,7 +869,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>45903.455555555556</v>
       </c>
@@ -890,7 +890,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>45903.463888888888</v>
       </c>
@@ -911,7 +911,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>45903.46597222222</v>
       </c>
@@ -932,7 +932,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>45903.467361111114</v>
       </c>
@@ -953,7 +953,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>45903.46875</v>
       </c>
@@ -974,7 +974,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>45903.470138888886</v>
       </c>
@@ -995,7 +995,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>45903.474999999999</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>45903.476388888892</v>
       </c>
@@ -1037,7 +1037,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>45903.479861111111</v>
       </c>
@@ -1058,7 +1058,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>45903.480555555558</v>
       </c>
@@ -1079,7 +1079,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>45903.493750000001</v>
       </c>
@@ -1100,7 +1100,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>45903.494444444441</v>
       </c>
@@ -1121,7 +1121,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>45903.494444444441</v>
       </c>
@@ -1142,7 +1142,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>45903.495138888888</v>
       </c>
@@ -1163,7 +1163,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>45903.504861111112</v>
       </c>
@@ -1184,7 +1184,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>45904.404861111114</v>
       </c>
@@ -1205,7 +1205,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>45904.406944444447</v>
       </c>
@@ -1226,7 +1226,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>45904.407638888886</v>
       </c>
@@ -1247,7 +1247,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>45904.412499999999</v>
       </c>
@@ -1268,7 +1268,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>45904.414583333331</v>
       </c>
@@ -1289,7 +1289,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>45904.418749999997</v>
       </c>
@@ -1310,7 +1310,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>45905.408333333333</v>
       </c>
@@ -1331,7 +1331,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>45908.665277777778</v>
       </c>
@@ -1352,7 +1352,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>45909.415277777778</v>
       </c>
@@ -1373,7 +1373,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>45909.418055555558</v>
       </c>
@@ -1394,7 +1394,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>45909.427083333336</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>45909.427777777775</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>45909.431250000001</v>
       </c>
@@ -1457,7 +1457,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>45909.43472222222</v>
       </c>
@@ -1478,7 +1478,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>45909.439583333333</v>
       </c>
@@ -1499,7 +1499,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>45909.449305555558</v>
       </c>
@@ -1520,7 +1520,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>45909.449305555558</v>
       </c>
@@ -1541,7 +1541,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>45910</v>
       </c>
@@ -1562,7 +1562,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>45910</v>
       </c>
@@ -1583,7 +1583,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>45911</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>45911</v>
       </c>
@@ -1625,7 +1625,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>45912</v>
       </c>
@@ -1646,7 +1646,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>45912</v>
       </c>
@@ -1667,7 +1667,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>45912</v>
       </c>
@@ -1688,7 +1688,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>45912</v>
       </c>
@@ -1709,7 +1709,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>45923</v>
       </c>
@@ -1730,7 +1730,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>45923</v>
       </c>
@@ -1751,7 +1751,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>45923</v>
       </c>
@@ -1772,7 +1772,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>45923</v>
       </c>
@@ -1793,7 +1793,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>45923</v>
       </c>
@@ -1814,7 +1814,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>45923</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>45924</v>
       </c>
@@ -1856,7 +1856,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>45924</v>
       </c>
@@ -1877,7 +1877,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>45929</v>
       </c>
@@ -1898,7 +1898,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>45937</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>45937</v>
       </c>
@@ -1940,7 +1940,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>45937</v>
       </c>
@@ -1961,7 +1961,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>45937.40625</v>
       </c>
@@ -1982,7 +1982,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>45937.462500000001</v>
       </c>
@@ -2003,7 +2003,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>45937.465277777781</v>
       </c>
@@ -2024,7 +2024,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>45938.413194444445</v>
       </c>
@@ -2044,7 +2044,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>45939.417361111111</v>
       </c>
@@ -2064,7 +2064,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>45943.410416666666</v>
       </c>
@@ -2084,7 +2084,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>45943.411805555559</v>
       </c>
@@ -2104,7 +2104,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>45943.412499999999</v>
       </c>
@@ -2124,7 +2124,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>45943.413194444445</v>
       </c>
@@ -2144,7 +2144,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>45943.415277777778</v>
       </c>
@@ -2164,7 +2164,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>45943.417361111111</v>
       </c>
@@ -2184,7 +2184,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>45946.399305555555</v>
       </c>
@@ -2204,7 +2204,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>45957.457638888889</v>
       </c>
@@ -2224,7 +2224,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>45957.459722222222</v>
       </c>
@@ -2244,7 +2244,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>45957.460416666669</v>
       </c>
@@ -2264,7 +2264,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>45957.462500000001</v>
       </c>
@@ -2284,7 +2284,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>45957.463194444441</v>
       </c>
@@ -2304,7 +2304,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>45957.463888888888</v>
       </c>
@@ -2324,7 +2324,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>45957.464583333334</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>45957.464583333334</v>
       </c>
@@ -2364,7 +2364,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>45957.470833333333</v>
       </c>
@@ -2384,7 +2384,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>45957.470833333333</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>45957.47152777778</v>
       </c>
@@ -2424,7 +2424,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>45958.512499999997</v>
       </c>
@@ -2444,7 +2444,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>45958.515277777777</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>45958.517361111109</v>
       </c>
@@ -2484,7 +2484,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>45958.520138888889</v>
       </c>
@@ -2504,7 +2504,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>45958.522222222222</v>
       </c>
@@ -2524,7 +2524,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <v>45958.522222222222</v>
       </c>
@@ -2544,7 +2544,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>45958.529166666667</v>
       </c>
@@ -2564,7 +2564,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>45965.642361111109</v>
       </c>
@@ -2584,7 +2584,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
         <v>45974.67291666667</v>
       </c>
@@ -2604,7 +2604,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>46002.439583333333</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>46002.443749999999</v>
       </c>
@@ -2644,7 +2644,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>46002.446527777778</v>
       </c>
@@ -2664,7 +2664,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>46008.648611111108</v>
       </c>
@@ -2684,7 +2684,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>46008.650694444441</v>
       </c>
@@ -2704,7 +2704,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>46020.463888888888</v>
       </c>
@@ -2724,7 +2724,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
         <v>46021.472916666666</v>
       </c>
@@ -2744,7 +2744,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
         <v>46027.567361111112</v>
       </c>
@@ -2764,7 +2764,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>46027.568055555559</v>
       </c>
@@ -2784,7 +2784,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
         <v>46027.568749999999</v>
       </c>
@@ -2804,7 +2804,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
         <v>46029.449305555558</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
         <v>46034.47152777778</v>
       </c>
@@ -2844,7 +2844,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="1">
         <v>46034.47152777778</v>
       </c>
@@ -2864,7 +2864,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
         <v>46035.44027777778</v>
       </c>
@@ -2884,7 +2884,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
         <v>46035.441666666666</v>
       </c>
@@ -2904,7 +2904,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
         <v>46036.448611111111</v>
       </c>
@@ -2924,7 +2924,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
         <v>46042.441666666666</v>
       </c>
@@ -2944,7 +2944,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="1">
         <v>46042.44027777778</v>
       </c>
@@ -2964,7 +2964,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
         <v>46042.45</v>
       </c>
@@ -2984,7 +2984,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="1">
         <v>46044.496527777781</v>
       </c>
@@ -3005,7 +3005,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
         <v>46044.496527777781</v>
       </c>
@@ -3025,7 +3025,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
         <v>46044.49722222222</v>
       </c>
@@ -3045,7 +3045,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
         <v>46045.445833333331</v>
       </c>
@@ -3065,7 +3065,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
         <v>46045.493055555555</v>
       </c>
@@ -3085,7 +3085,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
         <v>46048.572222222225</v>
       </c>
@@ -3105,7 +3105,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
         <v>46049.448611111111</v>
       </c>
@@ -3125,7 +3125,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" s="1">
         <v>46050.563888888886</v>
       </c>
@@ -3145,7 +3145,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
         <v>46059</v>
       </c>
@@ -3165,7 +3165,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" s="1">
         <v>46055.650694444441</v>
       </c>
@@ -3185,7 +3185,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" s="1">
         <v>46055.652083333334</v>
       </c>
@@ -3205,7 +3205,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" s="1">
         <v>46083.456250000003</v>
       </c>
@@ -3225,7 +3225,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="1">
         <v>46086</v>
       </c>
@@ -3245,7 +3245,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
         <v>46002</v>
       </c>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" s="1">
         <v>46087</v>
       </c>
@@ -3285,7 +3285,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" s="1">
         <v>46087</v>
       </c>
@@ -3305,7 +3305,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" s="1">
         <v>46087</v>
       </c>
@@ -3325,7 +3325,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" s="1">
         <v>46087</v>
       </c>
@@ -3345,7 +3345,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133" s="1">
         <v>46087</v>
       </c>
@@ -3365,7 +3365,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" s="1">
         <v>46087</v>
       </c>
@@ -3385,7 +3385,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135" s="1">
         <v>46087</v>
       </c>
@@ -3405,7 +3405,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" s="1">
         <v>46090</v>
       </c>
@@ -3425,7 +3425,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" s="1">
         <v>46090</v>
       </c>
@@ -3445,7 +3445,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" s="1">
         <v>46090</v>
       </c>
@@ -3465,7 +3465,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" s="1">
         <v>46090</v>
       </c>
@@ -3485,7 +3485,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" s="1">
         <v>46090</v>
       </c>
@@ -3505,7 +3505,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" s="1">
         <v>46091</v>
       </c>
@@ -3525,7 +3525,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" s="1">
         <v>46091</v>
       </c>
@@ -3545,7 +3545,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" s="1">
         <v>46091</v>
       </c>
@@ -3565,7 +3565,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" s="1">
         <v>46091</v>
       </c>
@@ -3585,7 +3585,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" s="1">
         <v>46091</v>
       </c>
@@ -3605,7 +3605,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146" s="1">
         <v>46092</v>
       </c>

</xml_diff>

<commit_message>
Update portfolio as of 2026-04-15
</commit_message>
<xml_diff>
--- a/data/portfolio_activity.xlsx
+++ b/data/portfolio_activity.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2018001\work_desktop\_personal\finance_portfolio\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5AC8212-F905-4291-B03B-D12169F7BD8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BECF0BE5-D668-45AD-AF70-049381FD0252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{22981F44-200C-FA48-B0C7-1CB3C862DEAA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="62">
   <si>
     <t>date</t>
   </si>
@@ -629,7 +629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64184D08-D91B-1043-AEE3-17C45FED0F30}">
-  <dimension ref="A1:F148"/>
+  <dimension ref="A1:F152"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.125" style="1" customWidth="1"/>
@@ -3666,6 +3666,86 @@
         <v>7</v>
       </c>
     </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A149" s="1">
+        <v>46113</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C149" s="6">
+        <v>1054.31</v>
+      </c>
+      <c r="D149" s="6">
+        <v>123.39</v>
+      </c>
+      <c r="E149" s="6">
+        <v>8.5441699999999994</v>
+      </c>
+      <c r="F149" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A150" s="1">
+        <v>46113</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C150" s="6">
+        <v>515.58000000000004</v>
+      </c>
+      <c r="D150" s="6">
+        <v>71.459999999999994</v>
+      </c>
+      <c r="E150" s="6">
+        <v>7.2149599999999996</v>
+      </c>
+      <c r="F150" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A151" s="1">
+        <v>46113</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C151" s="6">
+        <v>500</v>
+      </c>
+      <c r="D151" s="6">
+        <v>83.33</v>
+      </c>
+      <c r="E151" s="6">
+        <v>6.0002399999999998</v>
+      </c>
+      <c r="F151" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A152" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C152" s="6">
+        <v>715.9</v>
+      </c>
+      <c r="D152" s="6">
+        <v>371.51</v>
+      </c>
+      <c r="E152" s="6">
+        <v>1.927</v>
+      </c>
+      <c r="F152" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F128" xr:uid="{64184D08-D91B-1043-AEE3-17C45FED0F30}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add activities as of 2026-04-22
</commit_message>
<xml_diff>
--- a/data/portfolio_activity.xlsx
+++ b/data/portfolio_activity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2018001\work_desktop\_personal\finance_portfolio\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BECF0BE5-D668-45AD-AF70-049381FD0252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0017A1D-3F4C-494D-AF23-18D2C93F7C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{22981F44-200C-FA48-B0C7-1CB3C862DEAA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="63">
   <si>
     <t>date</t>
   </si>
@@ -225,6 +225,9 @@
   </si>
   <si>
     <t>RING</t>
+  </si>
+  <si>
+    <t>HOOD</t>
   </si>
 </sst>
 </file>
@@ -629,7 +632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64184D08-D91B-1043-AEE3-17C45FED0F30}">
-  <dimension ref="A1:F152"/>
+  <dimension ref="A1:F154"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.125" style="1" customWidth="1"/>
@@ -3746,6 +3749,46 @@
         <v>7</v>
       </c>
     </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A153" s="1">
+        <v>46128</v>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C153" s="6">
+        <v>638.77</v>
+      </c>
+      <c r="D153" s="6">
+        <v>86.03</v>
+      </c>
+      <c r="E153" s="6">
+        <v>7.42</v>
+      </c>
+      <c r="F153" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A154" s="1">
+        <v>46128</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C154" s="6">
+        <v>525.80999999999995</v>
+      </c>
+      <c r="D154" s="6">
+        <v>175.27</v>
+      </c>
+      <c r="E154" s="6">
+        <v>3</v>
+      </c>
+      <c r="F154" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F128" xr:uid="{64184D08-D91B-1043-AEE3-17C45FED0F30}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>